<commit_message>
big update, individual calendars, formatting
</commit_message>
<xml_diff>
--- a/input-output/Template.xlsx
+++ b/input-output/Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Scheduler\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Scheduler\input-output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4534F60E-B550-404A-93EB-91E5A7DC2E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C100CD5-08E5-4AA6-B4E1-DA04CBFB0DE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-32295" yWindow="4815" windowWidth="28800" windowHeight="15885" firstSheet="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="3210" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="edited" sheetId="1" r:id="rId1"/>
@@ -848,8 +848,8 @@
       <c r="E5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>19</v>
+      <c r="F5" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="G5" s="10" t="s">
         <v>22</v>
@@ -932,8 +932,12 @@
         <v>23</v>
       </c>
       <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
+      <c r="L6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>19</v>
+      </c>
       <c r="N6" s="5" t="s">
         <v>11</v>
       </c>
@@ -1188,8 +1192,8 @@
       <c r="E10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>19</v>
+      <c r="F10" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>19</v>
@@ -1479,12 +1483,6 @@
       </c>
       <c r="K14" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="L14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="M14" s="6" t="s">
-        <v>12</v>
       </c>
       <c r="N14" s="7" t="s">
         <v>19</v>
@@ -1774,7 +1772,6 @@
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
@@ -1827,7 +1824,6 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>

</xml_diff>